<commit_message>
commit inflows ratio calcs
</commit_message>
<xml_diff>
--- a/inflows_ny_dwelling_98_25.xlsx
+++ b/inflows_ny_dwelling_98_25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilnygaardeik/Documents/Industrial_Ecology/V_2026/MFA2/Project/TEP4290-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E5AB4F-F037-EC4B-B072-CB563BC5794F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99B7CD1-A50D-9E46-954A-32AAE8109266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -240,6 +240,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1598,7 +1599,7 @@
       <c r="C14" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="7">
         <f>AVERAGE(D9:AE9)</f>
         <v>1.7183886041235687E-2</v>
       </c>

</xml_diff>